<commit_message>
Update APB Timer IP: fix wait state, add cnt_behavior_chk, refresh docs
</commit_message>
<xml_diff>
--- a/apb_timer_ip/docs/VPLAN_TIMER_IP.xlsx
+++ b/apb_timer_ip/docs/VPLAN_TIMER_IP.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/72e3bfec65a6a2c0/Documents/Desktop/Vi_Mach/ICTC/Project/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/72e3bfec65a6a2c0/Documents/Desktop/Vi_Mach/Project/Project_Demo/design-verification-portfolio/apb_timer_ip/docs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="31" documentId="14_{A1D6CF54-4428-4D50-9673-9CE96EE3A2F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E02BB349-6523-4D55-BA48-9AE3D5AD6796}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{4C82EB97-2748-464C-91AB-8E5B25E09A2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{3587EFEC-8D9A-4C98-9936-48D5D12D96D6}"/>
   </bookViews>
@@ -901,11 +901,6 @@
     <t>Hardware Auto-Clear vs APB Write</t>
   </si>
   <si>
-    <t>Set timer_en = 1
-Write 0 to TCR.timer_en
-At the exact same clock cycle timer_en_fall asserts, use APB to write 0xFFFF_FFFF to TDR0.</t>
-  </si>
-  <si>
     <t>TCMP0/1</t>
   </si>
   <si>
@@ -922,17 +917,7 @@
 Interrupt asserts correctly when counter reaches 0xAAAA.</t>
   </si>
   <si>
-    <t>TDR0 is 32'h0000_0000 (Hardware Auto-Clear overrides APB Write)</t>
-  </si>
-  <si>
     <t>APB Write vs Hardware Increment</t>
-  </si>
-  <si>
-    <t>Set div_val = 0, timer_en = 1
-At the exact clock cycle the counter prepares to increment (+1), use APB to write 0xAAAA_AAAA to TDR0</t>
-  </si>
-  <si>
-    <t>TDR0 is 32'hAAAA_AAAA (APB Write overrides Hardware Increment)</t>
   </si>
   <si>
     <t>RW1C vs Hardware Set</t>
@@ -962,6 +947,28 @@
   </si>
   <si>
     <t>SUMMARY REPORT</t>
+  </si>
+  <si>
+    <t>Case A: TDR0 is 32'h5555_5555 (APB write after auto-clear is not lost).
+Case B: TDR0 and TDR1 are 32'h0000_0000 (HW auto-clear clears the counter).</t>
+  </si>
+  <si>
+    <t>1. Set div_en = 0 (counter increments every clock), timer_en = 1, wait 20 cycles.
+2. Write 0xAAAA_AAAA to TDR0 while the counter is running (the write collides with the HW increment).
+3. Read back TDR0 and TDR1.</t>
+  </si>
+  <si>
+    <t>1. Set timer_en = 1, wait some cycles.
+2. Write 0 to TCR.timer_en (timer_en falls, HW auto-clear is triggered).
+3. Case A: immediately issue an APB write of 0x5555_5555 to TDR0 (back-to-back, right after the TCR write). Read back TDR0.
+4. Case B: before step 2, write 0xAAAA_AAAA to TDR0. Then stop the timer as in step 2. Read back TDR0 and TDR1.
+Note: a same-cycle collision between timer_en_fall and an APB write cannot
+occur with a protocol-compliant APB master (min. 3 cycles per transfer,
+timer_en_fall lasts 1 cycle right after the TCR write completes).</t>
+  </si>
+  <si>
+    <t>TDR0 is in range [32'hAAAA_AAAA, 32'hAAAA_AAAA + 32] and TDR1 is 32'h0
+(APB Write overrides Hardware Increment, then counter keeps counting during the read latency).</t>
   </si>
 </sst>
 </file>
@@ -1181,12 +1188,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1197,6 +1198,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1235,10 +1242,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1624,10 +1627,10 @@
       <c r="H2" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J2" s="7" t="s">
-        <v>225</v>
-      </c>
-      <c r="K2" s="8"/>
+      <c r="J2" s="11" t="s">
+        <v>221</v>
+      </c>
+      <c r="K2" s="12"/>
     </row>
     <row r="3" spans="1:11" ht="72" x14ac:dyDescent="0.3">
       <c r="A3" s="2">
@@ -1650,10 +1653,10 @@
       <c r="H3" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J3" s="9" t="s">
-        <v>220</v>
-      </c>
-      <c r="K3" s="10">
+      <c r="J3" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="K3" s="8">
         <f>MAX(A2:A73)</f>
         <v>72</v>
       </c>
@@ -1679,10 +1682,10 @@
       <c r="H4" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J4" s="9" t="s">
-        <v>221</v>
-      </c>
-      <c r="K4" s="10">
+      <c r="J4" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="K4" s="8">
         <f>COUNTIFS($H$2:$H$73,"PASSED")</f>
         <v>72</v>
       </c>
@@ -1710,10 +1713,10 @@
       <c r="H5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J5" s="9" t="s">
-        <v>222</v>
-      </c>
-      <c r="K5" s="10">
+      <c r="J5" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="K5" s="8">
         <f>COUNTIFS($I$9:$I$76,"FAILED")</f>
         <v>0</v>
       </c>
@@ -1739,10 +1742,10 @@
       <c r="H6" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J6" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="K6" s="10">
+      <c r="J6" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="K6" s="8">
         <f>K3-(K4+K5)</f>
         <v>0</v>
       </c>
@@ -1768,10 +1771,10 @@
       <c r="H7" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="J7" s="11" t="s">
-        <v>224</v>
-      </c>
-      <c r="K7" s="12">
+      <c r="J7" s="9" t="s">
+        <v>220</v>
+      </c>
+      <c r="K7" s="10">
         <f>K4/K3*100</f>
         <v>100</v>
       </c>
@@ -1986,16 +1989,16 @@
       </c>
       <c r="B17" s="1"/>
       <c r="C17" s="2" t="s">
+        <v>208</v>
+      </c>
+      <c r="D17" s="2" t="s">
         <v>209</v>
       </c>
-      <c r="D17" s="2" t="s">
+      <c r="E17" s="1" t="s">
         <v>210</v>
       </c>
-      <c r="E17" s="1" t="s">
+      <c r="F17" s="1" t="s">
         <v>211</v>
-      </c>
-      <c r="F17" s="1" t="s">
-        <v>212</v>
       </c>
       <c r="G17" s="3" t="s">
         <v>18</v>
@@ -2438,7 +2441,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="37" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:8" ht="129.6" x14ac:dyDescent="0.3">
       <c r="A37" s="2">
         <v>36</v>
       </c>
@@ -2450,35 +2453,35 @@
         <v>207</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>208</v>
+        <v>224</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>213</v>
+        <v>222</v>
       </c>
       <c r="G37" s="1" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="H37" s="2" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="38" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A38" s="2">
         <v>37</v>
       </c>
       <c r="B38" s="1"/>
       <c r="C38" s="1"/>
       <c r="D38" s="1" t="s">
-        <v>214</v>
-      </c>
-      <c r="E38" s="3" t="s">
+        <v>212</v>
+      </c>
+      <c r="E38" s="2" t="s">
+        <v>223</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>225</v>
+      </c>
+      <c r="G38" s="1" t="s">
         <v>215</v>
-      </c>
-      <c r="F38" s="1" t="s">
-        <v>216</v>
-      </c>
-      <c r="G38" s="1" t="s">
-        <v>219</v>
       </c>
       <c r="H38" s="2" t="s">
         <v>14</v>
@@ -3277,10 +3280,10 @@
         <v>204</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="F73" s="1" t="s">
         <v>205</v>

</xml_diff>